<commit_message>
Deja en el PR solo los datos nuevos de Europa League
Las otras 7 ligas y validacion.json vuelven a la versión de main: los
actualiza el Action diario allí, así el PR no choca con esos archivos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CfurUCPh3W1YAk6TMxicy4
</commit_message>
<xml_diff>
--- a/datos/bbdd_laliga.xlsx
+++ b/datos/bbdd_laliga.xlsx
@@ -11,7 +11,7 @@
     <sheet name="diccionario" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'partidos'!$A$1:$AB$470</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'partidos'!$A$1:$AB$469</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB470"/>
+  <dimension ref="A1:AB469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -46483,106 +46483,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="470">
-      <c r="A470" s="2" t="inlineStr">
-        <is>
-          <t>2026-27</t>
-        </is>
-      </c>
-      <c r="B470" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="C470" s="2" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="D470" s="2" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="E470" s="2" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="F470" s="2" t="inlineStr">
-        <is>
-          <t>Levante</t>
-        </is>
-      </c>
-      <c r="G470" s="2" t="inlineStr">
-        <is>
-          <t>Athletic Club</t>
-        </is>
-      </c>
-      <c r="H470" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I470" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J470" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K470" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L470" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M470" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N470" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O470" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="P470" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q470" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="R470" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="S470" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="T470" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="U470" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="V470" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="W470" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="X470" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="Y470" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z470" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA470" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB470" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AB470"/>
+  <autoFilter ref="A1:AB469"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -46939,7 +46841,7 @@
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>469 partidos (2025-26: 380 partidos, 2026-27: 89 partidos). 28 columnas. Cargado el 22/10/2026.</t>
+          <t>468 partidos (2025-26: 380 partidos, 2026-27: 88 partidos). 28 columnas. Cargado el 21/10/2026.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">

</xml_diff>